<commit_message>
Updated paths for GL2 in Test file
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/TestGL2/ReferenceData/RefData_SBO_EVENTS.xlsx
+++ b/src/test/resources/TestDriver/TestGL2/ReferenceData/RefData_SBO_EVENTS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alijaffar/Documents/GitHub/fyntrac-data/src/test/resources/TestDriver/TestGL2/ReferenceData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alijaffar/workspace/fyntrac-data/src/test/resources/TestDriver/TestGL2/ReferenceData/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ECAAEB7-202A-D44C-A94C-FA4141E08887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37860" yWindow="1860" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Transactions" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Test driver: run long scenarios in pieces without re-dropping the tenant
- test.reset.database (default true) gates the tenant drop and fiscal-period
  seed; -PresetDb=false continues on the existing data.
- -PtestSteps=<file> selects the step workbook inside the testData folder.
- Hearst_GHK split into Test_P1 (config + Jun-Dec 2025, resets) and
  Test_P2..P4 (2026 in 4/2/2-month pieces); Test.xlsx kept for full runs.
- Driver logs tenant/steps/reset mode at startup.

Also includes pending Hearst_Ver/TestGL2 data updates and the new TestGLBase
folder that were in the working tree.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/TestGL2/ReferenceData/RefData_SBO_EVENTS.xlsx
+++ b/src/test/resources/TestDriver/TestGL2/ReferenceData/RefData_SBO_EVENTS.xlsx
@@ -1,41 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alijaffar/workspace/fyntrac-data/src/test/resources/TestDriver/TestGL2/ReferenceData/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ECAAEB7-202A-D44C-A94C-FA4141E08887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15860" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="Transactions" sheetId="1" r:id="rId1"/>
-    <sheet name="Attributes" sheetId="2" r:id="rId2"/>
-    <sheet name="Aggregation" sheetId="3" r:id="rId3"/>
-    <sheet name="AccountType" sheetId="4" r:id="rId4"/>
-    <sheet name="SubledgerMapping" sheetId="5" r:id="rId5"/>
-    <sheet name="ChartOfAccount" sheetId="6" r:id="rId6"/>
+    <sheet name="Transactions" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Attributes" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Aggregation" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="AccountType" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="SubledgerMapping" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="ChartOfAccount" sheetId="6" state="visible" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
@@ -43,36 +23,55 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>Unknown Author</author>
+    <author>tc={9E093D81-A130-42E7-B29A-6EA4F65C90AC}</author>
+    <author>tc={3EB65B76-479A-48D3-B5D2-FAFE57CE03F7}</author>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="C1" authorId="0" xr:uid="{9E093D81-A130-42E7-B29A-6EA4F65C90AC}">
       <text>
         <r>
           <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">Unknown Author:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">
+[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Controllable from UI as well, Settings&gt;Journal Fields, All booking attributes are reclassable</t>
+    Controllable from UI as well, Settings&gt;Journal Fields, All booking attributes are reclassable
+</t>
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+    <comment ref="D1" authorId="1" xr:uid="{3EB65B76-479A-48D3-B5D2-FAFE57CE03F7}">
       <text>
         <r>
           <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
           </rPr>
-          <t>[Threaded comment]
+          <t xml:space="preserve">Unknown Author:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">
+[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Controllable from UI as well, Settings&gt;Journal Fields, All booking attributes are reclassable</t>
+    Controllable from UI as well, Settings&gt;Journal Fields, All booking attributes are reclassable
+</t>
         </r>
       </text>
     </comment>
@@ -81,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t>Name</t>
   </si>
@@ -200,6 +199,9 @@
     <t>UserField9</t>
   </si>
   <si>
+    <t>PRODUCT_TYPE</t>
+  </si>
+  <si>
     <t>UserField10</t>
   </si>
   <si>
@@ -224,10 +226,16 @@
     <t>LAST_PAYMENT_MADE_DATE</t>
   </si>
   <si>
-    <t>Transaction Name</t>
-  </si>
-  <si>
-    <t>Metric Name</t>
+    <t>UserField14</t>
+  </si>
+  <si>
+    <t>PORTFOLIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transaction Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric Name</t>
   </si>
   <si>
     <t>Unpaid_Principal_Balance</t>
@@ -242,13 +250,13 @@
     <t>AccountType</t>
   </si>
   <si>
-    <t>Cash Receivable</t>
-  </si>
-  <si>
-    <t>Balance Sheet</t>
-  </si>
-  <si>
-    <t>Cash Clearing</t>
+    <t xml:space="preserve">Cash Receivable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balance Sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Clearing</t>
   </si>
   <si>
     <t>Clearing</t>
@@ -257,13 +265,13 @@
     <t>Principal</t>
   </si>
   <si>
-    <t>Interest Income</t>
-  </si>
-  <si>
-    <t>Income Statement</t>
-  </si>
-  <si>
-    <t>Accrued Interest Receivable</t>
+    <t xml:space="preserve">Interest Income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Income Statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accrued Interest Receivable</t>
   </si>
   <si>
     <t>TransactionName</t>
@@ -287,125 +295,93 @@
     <t>Credit</t>
   </si>
   <si>
-    <t>Account Name</t>
+    <t xml:space="preserve">Account Name</t>
   </si>
   <si>
     <t>AccountNumber</t>
   </si>
   <si>
-    <t>PRODUCT_TYPE</t>
-  </si>
-  <si>
-    <t>UserField14</t>
-  </si>
-  <si>
-    <t>PORTFOLIO</t>
+    <t xml:space="preserve">Cash Receivable 102</t>
   </si>
   <si>
     <t>ABC</t>
   </si>
   <si>
-    <t>Cash Receivable 102</t>
-  </si>
-  <si>
-    <t>Cash Clearing 102</t>
-  </si>
-  <si>
-    <t>Principal 102</t>
-  </si>
-  <si>
-    <t>Interest Income 102</t>
-  </si>
-  <si>
-    <t>Accrued Interest Receivable 102</t>
+    <t xml:space="preserve">Cash Clearing 102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Principal 102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interest Income 102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accrued Interest Receivable 102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Receivable 103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Clearing 103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Principal 103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interest Income 103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accrued Interest Receivable 103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Receivable 102R</t>
   </si>
   <si>
     <t>RAF</t>
   </si>
   <si>
-    <t>Cash Receivable 103</t>
-  </si>
-  <si>
-    <t>Cash Clearing 103</t>
-  </si>
-  <si>
-    <t>Principal 103</t>
-  </si>
-  <si>
-    <t>Interest Income 103</t>
-  </si>
-  <si>
-    <t>Accrued Interest Receivable 103</t>
-  </si>
-  <si>
-    <t>Cash Receivable 102R</t>
-  </si>
-  <si>
-    <t>Cash Clearing 102R</t>
-  </si>
-  <si>
-    <t>Principal 102R</t>
-  </si>
-  <si>
-    <t>Interest Income 102R</t>
-  </si>
-  <si>
-    <t>Accrued Interest Receivable 102R</t>
-  </si>
-  <si>
-    <t>Cash Receivable 103R</t>
-  </si>
-  <si>
-    <t>Cash Clearing 103R</t>
-  </si>
-  <si>
-    <t>Principal 103R</t>
-  </si>
-  <si>
-    <t>Interest Income 103R</t>
-  </si>
-  <si>
-    <t>Accrued Interest Receivable 103R</t>
+    <t xml:space="preserve">Cash Clearing 102R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Principal 102R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interest Income 102R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accrued Interest Receivable 102R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Receivable 103R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Clearing 103R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Principal 103R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interest Income 103R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accrued Interest Receivable 103R</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -417,27 +393,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor indexed="5"/>
+        <bgColor indexed="5"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="6">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="none"/>
+      <right style="none"/>
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -449,30 +425,30 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
-      <left/>
+      <left style="none"/>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right/>
+      <right style="none"/>
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -487,36 +463,36 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="12">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="1" applyFont="1"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="4" numFmtId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="1"/>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="5" numFmtId="0" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -531,8 +507,297 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Unknown Author" id="{BE284354-3A25-A9F4-8F97-E8617689BD3D}"/>
+</personList>
+</file>
+
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -574,17 +839,17 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -611,7 +876,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -635,7 +899,6 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -695,32 +958,50 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C1" personId="{BE284354-3A25-A9F4-8F97-E8617689BD3D}" id="{9E093D81-A130-42E7-B29A-6EA4F65C90AC}" done="0">
+    <text xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Controllable from UI as well, Settings&gt;Journal Fields, All booking attributes are reclassable
+</text>
+  </threadedComment>
+  <threadedComment ref="D1" personId="{BE284354-3A25-A9F4-8F97-E8617689BD3D}" id="{3EB65B76-479A-48D3-B5D2-FAFE57CE03F7}" done="0">
+    <text xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Controllable from UI as well, Settings&gt;Journal Fields, All booking attributes are reclassable
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor indexed="5"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="45.33203125" customWidth="1"/>
-    <col min="2" max="2" width="16.5" customWidth="1"/>
-    <col min="3" max="3" width="22.5" customWidth="1"/>
-    <col min="4" max="4" width="24.1640625" customWidth="1"/>
-    <col min="5" max="5" width="16.5" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="45.33203125"/>
+    <col customWidth="1" min="2" max="2" width="16.5"/>
+    <col customWidth="1" min="3" max="3" width="22.5"/>
+    <col customWidth="1" min="4" max="4" width="24.1640625"/>
+    <col customWidth="1" min="5" max="5" width="16.5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -734,7 +1015,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -748,7 +1029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -762,7 +1043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -776,7 +1057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -790,7 +1071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -804,7 +1085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -818,7 +1099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -832,7 +1113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -847,28 +1128,31 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor indexed="5"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="27.5" style="3" customWidth="1"/>
-    <col min="2" max="2" width="33.5" style="3" customWidth="1"/>
-    <col min="3" max="4" width="17" style="3" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" style="3"/>
-    <col min="6" max="6" width="10.5" style="3" customWidth="1"/>
-    <col min="7" max="16384" width="8.6640625" style="3"/>
+    <col customWidth="1" min="1" max="1" style="3" width="27.5"/>
+    <col customWidth="1" min="2" max="2" style="3" width="33.5"/>
+    <col customWidth="1" min="3" max="4" style="3" width="17"/>
+    <col min="5" max="5" style="3" width="8.6640625"/>
+    <col customWidth="1" min="6" max="6" style="3" width="10.5"/>
+    <col min="7" max="16384" style="3" width="8.6640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>12</v>
       </c>
@@ -888,7 +1172,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" s="3" t="s">
         <v>18</v>
       </c>
@@ -908,7 +1192,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3">
       <c r="A3" s="3" t="s">
         <v>22</v>
       </c>
@@ -928,7 +1212,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4" s="3" t="s">
         <v>25</v>
       </c>
@@ -948,7 +1232,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5">
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
@@ -968,7 +1252,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6">
       <c r="A6" s="3" t="s">
         <v>29</v>
       </c>
@@ -988,7 +1272,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7">
       <c r="A7" s="3" t="s">
         <v>32</v>
       </c>
@@ -1008,7 +1292,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8">
       <c r="A8" s="3" t="s">
         <v>34</v>
       </c>
@@ -1028,7 +1312,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9">
       <c r="A9" s="3" t="s">
         <v>36</v>
       </c>
@@ -1048,12 +1332,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10">
       <c r="A10" s="3" t="s">
         <v>38</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="C10" s="3">
         <v>1</v>
@@ -1068,12 +1352,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11">
       <c r="A11" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="3">
         <v>0</v>
@@ -1088,12 +1372,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12">
       <c r="A12" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" s="3">
         <v>0</v>
@@ -1108,12 +1392,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13">
       <c r="A13" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" s="3">
         <v>0</v>
@@ -1128,12 +1412,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14">
       <c r="A14" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" s="3">
         <v>0</v>
@@ -1148,12 +1432,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="C15" s="3">
         <v>1</v>
@@ -1169,90 +1453,93 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor indexed="5"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="67.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="24.6640625" style="3" customWidth="1"/>
-    <col min="3" max="16384" width="11.5" style="3"/>
+    <col customWidth="1" min="1" max="1" style="3" width="67.6640625"/>
+    <col customWidth="1" min="2" max="2" style="3" width="24.6640625"/>
+    <col min="3" max="16384" style="3" width="11.5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
@@ -1261,8 +1548,9 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
@@ -1271,69 +1559,71 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor indexed="5"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="39.5" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20" style="3" customWidth="1"/>
-    <col min="3" max="16384" width="11.5" style="3"/>
+    <col customWidth="1" min="1" max="1" style="3" width="39.5"/>
+    <col customWidth="1" min="2" max="2" style="3" width="20"/>
+    <col min="3" max="16384" style="3" width="11.5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
@@ -1342,233 +1632,247 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor indexed="5"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="67.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="11.5" style="3"/>
-    <col min="3" max="3" width="10.5" style="3" customWidth="1"/>
-    <col min="4" max="4" width="44.33203125" style="3" customWidth="1"/>
-    <col min="5" max="16384" width="11.5" style="3"/>
+    <col customWidth="1" min="1" max="1" style="3" width="67.6640625"/>
+    <col min="2" max="2" style="3" width="11.5"/>
+    <col customWidth="1" min="3" max="3" style="3" width="10.5"/>
+    <col customWidth="1" min="4" max="4" style="3" width="44.33203125"/>
+    <col min="5" max="16384" style="3" width="11.5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B2" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B3" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>66</v>
+      <c r="B4" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>69</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B5" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>66</v>
+      <c r="B6" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>69</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B7" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B8" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B9" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>66</v>
+      <c r="B10" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>69</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>66</v>
+      <c r="B12" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>69</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>53</v>
-      </c>
+      <c r="B15" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
@@ -1577,380 +1881,382 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor indexed="5"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5" style="3" customWidth="1"/>
-    <col min="2" max="2" width="16" style="3" customWidth="1"/>
-    <col min="3" max="3" width="39.5" style="3" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" style="3" customWidth="1"/>
-    <col min="5" max="16384" width="11.5" style="3"/>
+    <col customWidth="1" min="1" max="1" style="3" width="43.5"/>
+    <col customWidth="1" min="2" max="2" style="3" width="16"/>
+    <col customWidth="1" min="3" max="3" style="3" width="39.5"/>
+    <col customWidth="1" min="4" max="4" style="3" width="13.6640625"/>
+    <col min="5" max="16384" style="3" width="11.5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="E1" s="11" t="s">
+    <row r="1">
+      <c r="A1" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C1" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B2" s="9">
+        <v>73</v>
+      </c>
+      <c r="B2" s="10">
         <v>1000</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D2" s="3">
         <v>102</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>2000</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D3" s="3">
         <v>102</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>3000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D4" s="3">
         <v>102</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="10">
         <v>4000</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D5" s="3">
         <v>102</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>5000</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D6" s="3">
         <v>102</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="9">
+        <v>79</v>
+      </c>
+      <c r="B7" s="10">
         <v>6000</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D7" s="3">
         <v>103</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B8" s="9">
+        <v>80</v>
+      </c>
+      <c r="B8" s="10">
         <v>7000</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D8" s="3">
         <v>103</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B9" s="9">
+        <v>81</v>
+      </c>
+      <c r="B9" s="10">
         <v>8000</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D9" s="3">
         <v>103</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B10" s="9">
+        <v>82</v>
+      </c>
+      <c r="B10" s="10">
         <v>9000</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D10" s="3">
         <v>103</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="9">
+        <v>83</v>
+      </c>
+      <c r="B11" s="10">
         <v>10000</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D11" s="3">
         <v>103</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="9">
+        <v>84</v>
+      </c>
+      <c r="B12" s="10">
         <v>11000</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D12" s="3">
         <v>102</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>12000</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D13" s="3">
         <v>102</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>13000</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D14" s="3">
         <v>102</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="10">
         <v>14000</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D15" s="3">
         <v>102</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="10">
         <v>15000</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D16" s="3">
         <v>102</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="10">
         <v>16000</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D17" s="3">
         <v>103</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>17000</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D18" s="3">
         <v>103</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>18000</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D19" s="3">
         <v>103</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>19000</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D20" s="3">
         <v>103</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="10">
         <v>20000</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D21" s="3">
         <v>103</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>

</xml_diff>